<commit_message>
SF trip: v2 del presupuesto (nota sin '=' y etiqueta de total), nuevo link del Google Sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Travel/SF Sep-Nov 2026/Presupuesto SF Sep28-Nov4 2026.xlsx
+++ b/Travel/SF Sep-Nov 2026/Presupuesto SF Sep28-Nov4 2026.xlsx
@@ -1704,9 +1704,10 @@
           <t>USD/noche</t>
         </is>
       </c>
-      <c r="G9" s="5">
-        <f> unidad × tu parte.</f>
-        <v/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Unidad × tu parte (Supuestos B5).</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -4462,7 +4463,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>TOTAL VIAJE (sin vuelo)</t>
+          <t>TOTAL VIAJE (sin vuelo; lavandería y comidas con clientes solo en Resumen)</t>
         </is>
       </c>
       <c r="E43" s="12">

</xml_diff>